<commit_message>
Merge Hero Glamour models; add date range filter; remove Tracker tab
- Consolidate Hero Glamour X 125 into Hero Glamour in dashboard_data.json and cps_dashboard_updater.gs (MODEL_ALIAS map + normModel())
- Add From/To date range filter inputs to Daywise Analysis tab
- Remove Tracker tab button and panel from cps_dashboard_performance.html

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CV_Comparison.xlsx
+++ b/CV_Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deepanshi Ahuja\Desktop\Marketing_Performance_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AB68F4-FE03-4E9C-B248-BC28C6664D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333D2778-02D8-472C-8220-E4C14AE37FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{2A06160F-D6CF-40AF-81FB-3972BB152925}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="63">
   <si>
     <t>Spends</t>
   </si>
@@ -165,13 +165,83 @@
   </si>
   <si>
     <t>Aug'26</t>
+  </si>
+  <si>
+    <t>Enterprise</t>
+  </si>
+  <si>
+    <t>CPS</t>
+  </si>
+  <si>
+    <t>NCBD</t>
+  </si>
+  <si>
+    <t>Spend</t>
+  </si>
+  <si>
+    <t>Tleads</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Cars</t>
+  </si>
+  <si>
+    <t>Bikes</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Car</t>
+  </si>
+  <si>
+    <t>Bike</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>Q2'27</t>
+  </si>
+  <si>
+    <t>Trigger Leads</t>
+  </si>
+  <si>
+    <t>spend</t>
+  </si>
+  <si>
+    <t>rev</t>
+  </si>
+  <si>
+    <t>leads</t>
+  </si>
+  <si>
+    <t>tleads</t>
+  </si>
+  <si>
+    <t>t</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,19 +267,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -541,10 +616,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36EECC82-B786-4F88-BF54-40C3395F4A7F}">
-  <dimension ref="A1:AL30"/>
+  <dimension ref="A1:BN31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="45" max="47" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="9.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:66" x14ac:dyDescent="0.35">
       <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
@@ -595,7 +682,7 @@
       <c r="AK1" s="3"/>
       <c r="AL1" s="3"/>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -710,8 +797,44 @@
       <c r="AL2" t="s">
         <v>41</v>
       </c>
+      <c r="AS2">
+        <v>6777249</v>
+      </c>
+      <c r="AT2">
+        <v>112238</v>
+      </c>
+      <c r="AU2">
+        <v>60820</v>
+      </c>
+      <c r="AV2">
+        <f>AS2/AU2</f>
+        <v>111.43125616573495</v>
+      </c>
+      <c r="AX2">
+        <v>20500000</v>
+      </c>
+      <c r="AZ2" s="4">
+        <f>AVERAGE(AZ5,AZ8,AZ11)</f>
+        <v>2771773</v>
+      </c>
+      <c r="BA2" s="4">
+        <f>AVERAGE(BA5,BA8,BA11)</f>
+        <v>109176.66666666667</v>
+      </c>
+      <c r="BB2" s="4">
+        <f>AVERAGE(BB5,BB8,BB11)</f>
+        <v>70864</v>
+      </c>
+      <c r="BC2">
+        <f>AZ2/BA2</f>
+        <v>25.387961408115284</v>
+      </c>
+      <c r="BD2">
+        <f>AZ2/BB2</f>
+        <v>39.113978889139759</v>
+      </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -826,8 +949,26 @@
       <c r="AL3" s="2">
         <v>1</v>
       </c>
+      <c r="AS3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="3"/>
+      <c r="AV3" s="3"/>
+      <c r="AW3" s="3"/>
+      <c r="AX3" s="3"/>
+      <c r="AY3" s="3"/>
+      <c r="AZ3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="BA3" s="3"/>
+      <c r="BB3" s="3"/>
+      <c r="BC3" s="3"/>
+      <c r="BD3" s="3"/>
+      <c r="BE3" s="3"/>
+      <c r="BF3" s="3"/>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -942,8 +1083,62 @@
       <c r="AL4" s="2">
         <v>1</v>
       </c>
+      <c r="AS4" t="s">
+        <v>45</v>
+      </c>
+      <c r="AT4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AU4" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV4" t="s">
+        <v>2</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AX4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>5</v>
+      </c>
+      <c r="AZ4" t="s">
+        <v>45</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>1</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>46</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>2</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>4</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>47</v>
+      </c>
+      <c r="BF4" t="s">
+        <v>5</v>
+      </c>
+      <c r="BH4" t="s">
+        <v>58</v>
+      </c>
+      <c r="BI4" t="s">
+        <v>59</v>
+      </c>
+      <c r="BJ4" t="s">
+        <v>60</v>
+      </c>
+      <c r="BK4" t="s">
+        <v>61</v>
+      </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1058,8 +1253,81 @@
       <c r="AL5" s="2">
         <v>0.25</v>
       </c>
+      <c r="AQ5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS5" s="4">
+        <v>6000949</v>
+      </c>
+      <c r="AT5" s="4">
+        <v>88215</v>
+      </c>
+      <c r="AU5" s="4">
+        <v>60948</v>
+      </c>
+      <c r="AV5">
+        <f>AS5/AT5</f>
+        <v>68.026401405656628</v>
+      </c>
+      <c r="AW5">
+        <f>AS5/AU5</f>
+        <v>98.460146354269213</v>
+      </c>
+      <c r="AX5" s="4">
+        <v>14850434</v>
+      </c>
+      <c r="AY5" s="5">
+        <f>1-AS5/AX5</f>
+        <v>0.59590750007710214</v>
+      </c>
+      <c r="AZ5" s="4">
+        <v>2925953</v>
+      </c>
+      <c r="BA5" s="4">
+        <v>106863</v>
+      </c>
+      <c r="BB5" s="4">
+        <v>70949</v>
+      </c>
+      <c r="BC5">
+        <f>AZ5/BA5</f>
+        <v>27.380412303603681</v>
+      </c>
+      <c r="BD5">
+        <f>AZ5/BB5</f>
+        <v>41.240228896813207</v>
+      </c>
+      <c r="BE5" s="4">
+        <v>7549566</v>
+      </c>
+      <c r="BF5" s="5">
+        <f>1-AZ5/BE5</f>
+        <v>0.61243427767900838</v>
+      </c>
+      <c r="BG5" t="s">
+        <v>42</v>
+      </c>
+      <c r="BH5" s="4">
+        <f>AZ5+AS5</f>
+        <v>8926902</v>
+      </c>
+      <c r="BI5" s="4">
+        <f>BE5+AX5</f>
+        <v>22400000</v>
+      </c>
+      <c r="BJ5" s="4">
+        <f>BA5+AT5</f>
+        <v>195078</v>
+      </c>
+      <c r="BK5" s="4">
+        <f>BB5+AU5</f>
+        <v>131897</v>
+      </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1174,8 +1442,80 @@
       <c r="AL6" s="2">
         <v>0.17</v>
       </c>
+      <c r="AQ6" s="3"/>
+      <c r="AR6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS6" s="4">
+        <v>683700</v>
+      </c>
+      <c r="AT6" s="4">
+        <v>16228</v>
+      </c>
+      <c r="AU6">
+        <v>5779</v>
+      </c>
+      <c r="AV6">
+        <f t="shared" ref="AV6:AV13" si="0">AS6/AT6</f>
+        <v>42.130884890313041</v>
+      </c>
+      <c r="AW6">
+        <f t="shared" ref="AW6:AW13" si="1">AS6/AU6</f>
+        <v>118.30766568610487</v>
+      </c>
+      <c r="AX6" s="4">
+        <v>2504000</v>
+      </c>
+      <c r="AY6" s="5">
+        <f>1-AS6/AX6</f>
+        <v>0.72695686900958467</v>
+      </c>
+      <c r="AZ6" s="4">
+        <f>9974344+142771</f>
+        <v>10117115</v>
+      </c>
+      <c r="BA6">
+        <v>352904</v>
+      </c>
+      <c r="BB6">
+        <v>213026</v>
+      </c>
+      <c r="BC6">
+        <f t="shared" ref="BC6:BD13" si="2">AZ6/BA6</f>
+        <v>28.668178881508851</v>
+      </c>
+      <c r="BD6">
+        <f t="shared" ref="BD6:BD13" si="3">AZ6/BB6</f>
+        <v>47.492395294471095</v>
+      </c>
+      <c r="BE6">
+        <v>37199408</v>
+      </c>
+      <c r="BF6" s="5">
+        <f t="shared" ref="BF6:BF12" si="4">1-AZ6/BE6</f>
+        <v>0.72803021488944131</v>
+      </c>
+      <c r="BG6" t="s">
+        <v>43</v>
+      </c>
+      <c r="BH6" s="4">
+        <f t="shared" ref="BH6:BH13" si="5">AZ6+AS6</f>
+        <v>10800815</v>
+      </c>
+      <c r="BI6" s="4">
+        <f t="shared" ref="BI6:BI13" si="6">BE6+AX6</f>
+        <v>39703408</v>
+      </c>
+      <c r="BJ6" s="4">
+        <f t="shared" ref="BJ6:BJ13" si="7">BA6+AT6</f>
+        <v>369132</v>
+      </c>
+      <c r="BK6" s="4">
+        <f t="shared" ref="BK6:BK13" si="8">BB6+AU6</f>
+        <v>218805</v>
+      </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1290,8 +1630,73 @@
       <c r="AL7" s="2">
         <v>0.14000000000000001</v>
       </c>
+      <c r="AQ7" s="3"/>
+      <c r="AR7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AS7" s="4">
+        <v>3312566</v>
+      </c>
+      <c r="AT7" s="4">
+        <v>120078</v>
+      </c>
+      <c r="AU7" s="4">
+        <v>56760</v>
+      </c>
+      <c r="AV7">
+        <f t="shared" si="0"/>
+        <v>27.586785256250103</v>
+      </c>
+      <c r="AW7">
+        <f t="shared" si="1"/>
+        <v>58.36092318534179</v>
+      </c>
+      <c r="AX7" s="4">
+        <v>9575633</v>
+      </c>
+      <c r="AY7" s="5">
+        <f>1-AS7/AX7</f>
+        <v>0.65406297421799686</v>
+      </c>
+      <c r="AZ7">
+        <v>0</v>
+      </c>
+      <c r="BA7">
+        <v>0</v>
+      </c>
+      <c r="BC7" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BD7" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BF7" s="5" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BG7" t="s">
+        <v>44</v>
+      </c>
+      <c r="BH7" s="4">
+        <f t="shared" si="5"/>
+        <v>3312566</v>
+      </c>
+      <c r="BI7" s="4">
+        <f t="shared" si="6"/>
+        <v>9575633</v>
+      </c>
+      <c r="BJ7" s="4">
+        <f t="shared" si="7"/>
+        <v>120078</v>
+      </c>
+      <c r="BK7" s="4">
+        <f t="shared" si="8"/>
+        <v>56760</v>
+      </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1406,8 +1811,83 @@
       <c r="AL8" s="2">
         <v>0.14000000000000001</v>
       </c>
+      <c r="AQ8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS8" s="4">
+        <v>7459594</v>
+      </c>
+      <c r="AT8" s="4">
+        <v>132358</v>
+      </c>
+      <c r="AU8" s="4">
+        <v>63785</v>
+      </c>
+      <c r="AV8">
+        <f t="shared" si="0"/>
+        <v>56.359222714154036</v>
+      </c>
+      <c r="AW8">
+        <f t="shared" si="1"/>
+        <v>116.94903190405267</v>
+      </c>
+      <c r="AX8" s="4">
+        <v>15591320</v>
+      </c>
+      <c r="AY8" s="5">
+        <f>1-AS8/AX8</f>
+        <v>0.52155468555580931</v>
+      </c>
+      <c r="AZ8" s="4">
+        <f>1630221+215266</f>
+        <v>1845487</v>
+      </c>
+      <c r="BA8" s="4">
+        <v>72196</v>
+      </c>
+      <c r="BB8" s="4">
+        <v>43115</v>
+      </c>
+      <c r="BC8">
+        <f t="shared" si="2"/>
+        <v>25.562177959997783</v>
+      </c>
+      <c r="BD8">
+        <f t="shared" si="3"/>
+        <v>42.803826974370871</v>
+      </c>
+      <c r="BE8" s="4">
+        <f>AX2-AX8</f>
+        <v>4908680</v>
+      </c>
+      <c r="BF8" s="5">
+        <f t="shared" si="4"/>
+        <v>0.62403599338314986</v>
+      </c>
+      <c r="BG8" t="s">
+        <v>42</v>
+      </c>
+      <c r="BH8" s="4">
+        <f t="shared" si="5"/>
+        <v>9305081</v>
+      </c>
+      <c r="BI8" s="4">
+        <f t="shared" si="6"/>
+        <v>20500000</v>
+      </c>
+      <c r="BJ8" s="4">
+        <f t="shared" si="7"/>
+        <v>204554</v>
+      </c>
+      <c r="BK8" s="4">
+        <f t="shared" si="8"/>
+        <v>106900</v>
+      </c>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1522,8 +2002,79 @@
       <c r="AL9" s="2">
         <v>0.23</v>
       </c>
+      <c r="AQ9" s="3"/>
+      <c r="AR9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS9" s="4">
+        <v>701311</v>
+      </c>
+      <c r="AT9" s="4">
+        <v>17282</v>
+      </c>
+      <c r="AU9">
+        <v>8594</v>
+      </c>
+      <c r="AV9">
+        <f t="shared" si="0"/>
+        <v>40.580430505728501</v>
+      </c>
+      <c r="AW9">
+        <f t="shared" si="1"/>
+        <v>81.604724226204326</v>
+      </c>
+      <c r="AX9" s="4">
+        <v>2392000</v>
+      </c>
+      <c r="AY9" s="5">
+        <f>1-AS9/AX9</f>
+        <v>0.70680978260869565</v>
+      </c>
+      <c r="AZ9" s="4">
+        <v>11670404</v>
+      </c>
+      <c r="BA9">
+        <v>279941</v>
+      </c>
+      <c r="BB9">
+        <v>275758</v>
+      </c>
+      <c r="BC9">
+        <f t="shared" si="2"/>
+        <v>41.688798711156991</v>
+      </c>
+      <c r="BD9">
+        <f t="shared" si="3"/>
+        <v>42.321180165217328</v>
+      </c>
+      <c r="BE9">
+        <v>43138426</v>
+      </c>
+      <c r="BF9" s="5">
+        <f t="shared" si="4"/>
+        <v>0.7294661608654891</v>
+      </c>
+      <c r="BG9" t="s">
+        <v>43</v>
+      </c>
+      <c r="BH9" s="4">
+        <f t="shared" si="5"/>
+        <v>12371715</v>
+      </c>
+      <c r="BI9" s="4">
+        <f t="shared" si="6"/>
+        <v>45530426</v>
+      </c>
+      <c r="BJ9" s="4">
+        <f t="shared" si="7"/>
+        <v>297223</v>
+      </c>
+      <c r="BK9" s="4">
+        <f t="shared" si="8"/>
+        <v>284352</v>
+      </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1638,8 +2189,73 @@
       <c r="AL10" s="2">
         <v>0.23</v>
       </c>
+      <c r="AQ10" s="3"/>
+      <c r="AR10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AS10" s="4">
+        <v>4963294</v>
+      </c>
+      <c r="AT10" s="4">
+        <v>87495</v>
+      </c>
+      <c r="AU10">
+        <v>66155</v>
+      </c>
+      <c r="AV10">
+        <f t="shared" si="0"/>
+        <v>56.726601520086859</v>
+      </c>
+      <c r="AW10">
+        <f t="shared" si="1"/>
+        <v>75.025228629733206</v>
+      </c>
+      <c r="AX10" s="4">
+        <v>11839709</v>
+      </c>
+      <c r="AY10" s="5">
+        <f>1-AS10/AX10</f>
+        <v>0.58079256846599869</v>
+      </c>
+      <c r="AZ10" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA10">
+        <v>0</v>
+      </c>
+      <c r="BC10" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BD10" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BF10" s="5" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BG10" t="s">
+        <v>44</v>
+      </c>
+      <c r="BH10" s="4">
+        <f t="shared" si="5"/>
+        <v>4963294</v>
+      </c>
+      <c r="BI10" s="4">
+        <f t="shared" si="6"/>
+        <v>11839709</v>
+      </c>
+      <c r="BJ10" s="4">
+        <f t="shared" si="7"/>
+        <v>87495</v>
+      </c>
+      <c r="BK10" s="4">
+        <f t="shared" si="8"/>
+        <v>66155</v>
+      </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1754,8 +2370,81 @@
       <c r="AL11" s="2">
         <v>0.1</v>
       </c>
+      <c r="AQ11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS11" s="4">
+        <v>6871204</v>
+      </c>
+      <c r="AT11" s="4">
+        <v>116141</v>
+      </c>
+      <c r="AU11" s="4">
+        <v>57727</v>
+      </c>
+      <c r="AV11">
+        <f t="shared" si="0"/>
+        <v>59.162604076079937</v>
+      </c>
+      <c r="AW11">
+        <f t="shared" si="1"/>
+        <v>119.0292930517782</v>
+      </c>
+      <c r="AX11" s="4">
+        <v>13289218</v>
+      </c>
+      <c r="AY11" s="5">
+        <f>1-AS11/AX11</f>
+        <v>0.48294895907343838</v>
+      </c>
+      <c r="AZ11" s="4">
+        <v>3543879</v>
+      </c>
+      <c r="BA11" s="4">
+        <v>148471</v>
+      </c>
+      <c r="BB11" s="4">
+        <v>98528</v>
+      </c>
+      <c r="BC11">
+        <f t="shared" si="2"/>
+        <v>23.869166369189944</v>
+      </c>
+      <c r="BD11">
+        <f t="shared" si="3"/>
+        <v>35.968242530042218</v>
+      </c>
+      <c r="BE11" s="4">
+        <v>10073955</v>
+      </c>
+      <c r="BF11" s="5">
+        <f t="shared" si="4"/>
+        <v>0.64821373532043769</v>
+      </c>
+      <c r="BG11" t="s">
+        <v>42</v>
+      </c>
+      <c r="BH11" s="4">
+        <f t="shared" si="5"/>
+        <v>10415083</v>
+      </c>
+      <c r="BI11" s="4">
+        <f t="shared" si="6"/>
+        <v>23363173</v>
+      </c>
+      <c r="BJ11" s="4">
+        <f t="shared" si="7"/>
+        <v>264612</v>
+      </c>
+      <c r="BK11" s="4">
+        <f t="shared" si="8"/>
+        <v>156255</v>
+      </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1870,8 +2559,80 @@
       <c r="AL12" s="2">
         <v>0.1</v>
       </c>
+      <c r="AQ12" s="3"/>
+      <c r="AR12" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS12" s="4">
+        <v>718048</v>
+      </c>
+      <c r="AT12" s="4">
+        <v>14245</v>
+      </c>
+      <c r="AU12">
+        <v>8000</v>
+      </c>
+      <c r="AV12">
+        <f t="shared" si="0"/>
+        <v>50.407020007020009</v>
+      </c>
+      <c r="AW12">
+        <f t="shared" si="1"/>
+        <v>89.756</v>
+      </c>
+      <c r="AX12" s="4">
+        <v>2103000</v>
+      </c>
+      <c r="AY12" s="5">
+        <f>1-AS12/AX12</f>
+        <v>0.65856015216357577</v>
+      </c>
+      <c r="AZ12" s="4">
+        <f>15681336+262865</f>
+        <v>15944201</v>
+      </c>
+      <c r="BA12">
+        <v>272999</v>
+      </c>
+      <c r="BB12">
+        <v>297673</v>
+      </c>
+      <c r="BC12">
+        <f t="shared" si="2"/>
+        <v>58.403880600295238</v>
+      </c>
+      <c r="BD12">
+        <f t="shared" si="3"/>
+        <v>53.562805494619937</v>
+      </c>
+      <c r="BE12">
+        <v>32083992</v>
+      </c>
+      <c r="BF12" s="5">
+        <f t="shared" si="4"/>
+        <v>0.50304809326719691</v>
+      </c>
+      <c r="BG12" t="s">
+        <v>43</v>
+      </c>
+      <c r="BH12" s="4">
+        <f t="shared" si="5"/>
+        <v>16662249</v>
+      </c>
+      <c r="BI12" s="4">
+        <f t="shared" si="6"/>
+        <v>34186992</v>
+      </c>
+      <c r="BJ12" s="4">
+        <f t="shared" si="7"/>
+        <v>287244</v>
+      </c>
+      <c r="BK12" s="4">
+        <f t="shared" si="8"/>
+        <v>305673</v>
+      </c>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1986,8 +2747,69 @@
       <c r="AL13" s="2">
         <v>0.13</v>
       </c>
+      <c r="AQ13" s="3"/>
+      <c r="AR13" t="s">
+        <v>44</v>
+      </c>
+      <c r="AS13" s="4">
+        <v>3222804</v>
+      </c>
+      <c r="AT13" s="4">
+        <v>66637</v>
+      </c>
+      <c r="AU13">
+        <v>57000</v>
+      </c>
+      <c r="AV13">
+        <f t="shared" si="0"/>
+        <v>48.363581793898284</v>
+      </c>
+      <c r="AW13">
+        <f t="shared" si="1"/>
+        <v>56.540421052631579</v>
+      </c>
+      <c r="AX13" s="4">
+        <v>10578862</v>
+      </c>
+      <c r="AY13" s="5">
+        <f>1-AS13/AX13</f>
+        <v>0.69535437743681694</v>
+      </c>
+      <c r="AZ13" s="4">
+        <v>0</v>
+      </c>
+      <c r="BA13">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BD13" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="BG13" t="s">
+        <v>44</v>
+      </c>
+      <c r="BH13" s="4">
+        <f t="shared" si="5"/>
+        <v>3222804</v>
+      </c>
+      <c r="BI13" s="4">
+        <f t="shared" si="6"/>
+        <v>10578862</v>
+      </c>
+      <c r="BJ13" s="4">
+        <f t="shared" si="7"/>
+        <v>66637</v>
+      </c>
+      <c r="BK13" s="4">
+        <f t="shared" si="8"/>
+        <v>57000</v>
+      </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -2103,7 +2925,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -2218,8 +3040,35 @@
       <c r="AL15" s="2">
         <v>0.17</v>
       </c>
+      <c r="AS15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT15" s="3"/>
+      <c r="AU15" s="3"/>
+      <c r="AV15" s="3"/>
+      <c r="AW15" s="3"/>
+      <c r="AX15" s="3"/>
+      <c r="AY15" s="3"/>
+      <c r="AZ15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="BA15" s="3"/>
+      <c r="BB15" s="3"/>
+      <c r="BC15" s="3"/>
+      <c r="BD15" s="3"/>
+      <c r="BE15" s="3"/>
+      <c r="BF15" s="3"/>
+      <c r="BL15" t="s">
+        <v>56</v>
+      </c>
+      <c r="BM15" t="s">
+        <v>2</v>
+      </c>
+      <c r="BN15" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -2334,8 +3183,76 @@
       <c r="AL16" s="2">
         <v>0.14000000000000001</v>
       </c>
+      <c r="AR16" t="s">
+        <v>50</v>
+      </c>
+      <c r="AS16" s="4">
+        <f>SUM(AS5:AS7)</f>
+        <v>9997215</v>
+      </c>
+      <c r="AT16" s="4">
+        <f>SUM(AT5:AT7)</f>
+        <v>224521</v>
+      </c>
+      <c r="AU16" s="4">
+        <f>SUM(AU5:AU7)</f>
+        <v>123487</v>
+      </c>
+      <c r="AV16">
+        <f t="shared" ref="AV16:AV18" si="9">AS16/AT16</f>
+        <v>44.526859402906631</v>
+      </c>
+      <c r="AW16">
+        <f t="shared" ref="AW16:AW18" si="10">AS16/AU16</f>
+        <v>80.957631167653275</v>
+      </c>
+      <c r="AX16" s="4">
+        <f>SUM(AX5:AX7)</f>
+        <v>26930067</v>
+      </c>
+      <c r="AY16" s="5">
+        <f t="shared" ref="AY16:AY18" si="11">1-AS16/AX16</f>
+        <v>0.62877125407820189</v>
+      </c>
+      <c r="AZ16" s="4">
+        <f>SUM(AZ5:AZ7)</f>
+        <v>13043068</v>
+      </c>
+      <c r="BA16" s="4">
+        <f>SUM(BA5:BA7)</f>
+        <v>459767</v>
+      </c>
+      <c r="BB16" s="4">
+        <f>SUM(BB5:BB7)</f>
+        <v>283975</v>
+      </c>
+      <c r="BC16">
+        <f t="shared" ref="BC16:BD18" si="12">AZ16/BA16</f>
+        <v>28.368865099061047</v>
+      </c>
+      <c r="BD16">
+        <f t="shared" ref="BD16:BD18" si="13">AZ16/BB16</f>
+        <v>45.930338938286823</v>
+      </c>
+      <c r="BE16" s="4">
+        <f>SUM(BE5:BE7)</f>
+        <v>44748974</v>
+      </c>
+      <c r="BF16" s="5">
+        <f t="shared" ref="BF16:BF18" si="14">1-AZ16/BE16</f>
+        <v>0.70852811061098286</v>
+      </c>
+      <c r="BL16" t="s">
+        <v>48</v>
+      </c>
+      <c r="BM16" s="6">
+        <v>60.382838254423632</v>
+      </c>
+      <c r="BN16" s="6">
+        <v>111.43125616573495</v>
+      </c>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -2450,8 +3367,76 @@
       <c r="AL17" s="2">
         <v>0.14000000000000001</v>
       </c>
+      <c r="AR17" t="s">
+        <v>51</v>
+      </c>
+      <c r="AS17" s="4">
+        <f>SUM(AS8:AS10)</f>
+        <v>13124199</v>
+      </c>
+      <c r="AT17" s="4">
+        <f>SUM(AT8:AT10)</f>
+        <v>237135</v>
+      </c>
+      <c r="AU17" s="4">
+        <f>SUM(AU8:AU10)</f>
+        <v>138534</v>
+      </c>
+      <c r="AV17">
+        <f t="shared" si="9"/>
+        <v>55.344841545954836</v>
+      </c>
+      <c r="AW17">
+        <f t="shared" si="10"/>
+        <v>94.736303001429249</v>
+      </c>
+      <c r="AX17" s="4">
+        <f>SUM(AX8:AX10)</f>
+        <v>29823029</v>
+      </c>
+      <c r="AY17" s="5">
+        <f t="shared" si="11"/>
+        <v>0.55993071662841487</v>
+      </c>
+      <c r="AZ17" s="4">
+        <f>SUM(AZ8:AZ10)</f>
+        <v>13515891</v>
+      </c>
+      <c r="BA17" s="4">
+        <f>SUM(BA8:BA10)</f>
+        <v>352137</v>
+      </c>
+      <c r="BB17" s="4">
+        <f>SUM(BB8:BB10)</f>
+        <v>318873</v>
+      </c>
+      <c r="BC17">
+        <f t="shared" si="12"/>
+        <v>38.382478978352175</v>
+      </c>
+      <c r="BD17">
+        <f t="shared" si="13"/>
+        <v>42.386439115259051</v>
+      </c>
+      <c r="BE17" s="4">
+        <f>SUM(BE8:BE10)</f>
+        <v>48047106</v>
+      </c>
+      <c r="BF17" s="5">
+        <f t="shared" si="14"/>
+        <v>0.71869500319124313</v>
+      </c>
+      <c r="BL17" t="s">
+        <v>49</v>
+      </c>
+      <c r="BM17" s="6">
+        <v>25.387961408115284</v>
+      </c>
+      <c r="BN17" s="6">
+        <v>39.113978889139759</v>
+      </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -2566,8 +3551,67 @@
       <c r="AL18" s="2">
         <v>0.37</v>
       </c>
+      <c r="AR18" t="s">
+        <v>52</v>
+      </c>
+      <c r="AS18" s="4">
+        <f>SUM(AS11:AS13)</f>
+        <v>10812056</v>
+      </c>
+      <c r="AT18" s="4">
+        <f>SUM(AT11:AT13)</f>
+        <v>197023</v>
+      </c>
+      <c r="AU18" s="4">
+        <f>SUM(AU11:AU13)</f>
+        <v>122727</v>
+      </c>
+      <c r="AV18">
+        <f t="shared" si="9"/>
+        <v>54.877126020819901</v>
+      </c>
+      <c r="AW18">
+        <f t="shared" si="10"/>
+        <v>88.098429848362628</v>
+      </c>
+      <c r="AX18" s="4">
+        <f>SUM(AX11:AX13)</f>
+        <v>25971080</v>
+      </c>
+      <c r="AY18" s="5">
+        <f t="shared" si="11"/>
+        <v>0.58368862596395688</v>
+      </c>
+      <c r="AZ18" s="4">
+        <f>SUM(AZ11:AZ13)</f>
+        <v>19488080</v>
+      </c>
+      <c r="BA18" s="4">
+        <f>SUM(BA11:BA13)</f>
+        <v>421470</v>
+      </c>
+      <c r="BB18" s="4">
+        <f>SUM(BB11:BB13)</f>
+        <v>396201</v>
+      </c>
+      <c r="BC18">
+        <f t="shared" si="12"/>
+        <v>46.23835622938762</v>
+      </c>
+      <c r="BD18">
+        <f t="shared" si="13"/>
+        <v>49.187356922370213</v>
+      </c>
+      <c r="BE18" s="4">
+        <f>SUM(BE11:BE13)</f>
+        <v>42157947</v>
+      </c>
+      <c r="BF18" s="5">
+        <f t="shared" si="14"/>
+        <v>0.53773650315562094</v>
+      </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -2683,7 +3727,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -2798,8 +3842,31 @@
       <c r="AL20" s="2">
         <v>0.09</v>
       </c>
+      <c r="AT20" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AV20" t="s">
+        <v>5</v>
+      </c>
+      <c r="BB20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="BC20" s="3"/>
+      <c r="BD20" s="3"/>
+      <c r="BE20" s="3"/>
+      <c r="BF20" s="3"/>
+      <c r="BG20" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="BH20" s="3"/>
+      <c r="BI20" s="3"/>
+      <c r="BJ20" s="3"/>
+      <c r="BK20" s="3"/>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2914,8 +3981,53 @@
       <c r="AL21" s="2">
         <v>0.1</v>
       </c>
+      <c r="AS21" t="s">
+        <v>55</v>
+      </c>
+      <c r="AT21" s="4">
+        <f>SUM(AS16,AZ16)</f>
+        <v>23040283</v>
+      </c>
+      <c r="AU21" s="4">
+        <f>SUM(AX16,BE16)</f>
+        <v>71679041</v>
+      </c>
+      <c r="AV21" s="5">
+        <f>1-AT21/AU21</f>
+        <v>0.67856317999566984</v>
+      </c>
+      <c r="BB21" t="s">
+        <v>45</v>
+      </c>
+      <c r="BC21" t="s">
+        <v>1</v>
+      </c>
+      <c r="BD21" t="s">
+        <v>57</v>
+      </c>
+      <c r="BE21" t="s">
+        <v>2</v>
+      </c>
+      <c r="BF21" t="s">
+        <v>4</v>
+      </c>
+      <c r="BG21" t="s">
+        <v>45</v>
+      </c>
+      <c r="BH21" t="s">
+        <v>1</v>
+      </c>
+      <c r="BI21" t="s">
+        <v>57</v>
+      </c>
+      <c r="BJ21" t="s">
+        <v>2</v>
+      </c>
+      <c r="BK21" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -3030,8 +4142,58 @@
       <c r="AL22" s="2">
         <v>0</v>
       </c>
+      <c r="AS22" t="s">
+        <v>51</v>
+      </c>
+      <c r="AT22" s="4">
+        <f t="shared" ref="AT22:AT23" si="15">SUM(AS17,AZ17)</f>
+        <v>26640090</v>
+      </c>
+      <c r="AU22" s="4">
+        <f t="shared" ref="AU22:AU23" si="16">SUM(AX17,BE17)</f>
+        <v>77870135</v>
+      </c>
+      <c r="AV22" s="5">
+        <f t="shared" ref="AV22:AV25" si="17">1-AT22/AU22</f>
+        <v>0.65789079471866851</v>
+      </c>
+      <c r="BA22" t="s">
+        <v>50</v>
+      </c>
+      <c r="BB22">
+        <v>9997215</v>
+      </c>
+      <c r="BC22">
+        <v>224521</v>
+      </c>
+      <c r="BD22">
+        <v>123487</v>
+      </c>
+      <c r="BE22" s="6">
+        <v>44.526859402906631</v>
+      </c>
+      <c r="BF22" s="6">
+        <v>80.957631167653275</v>
+      </c>
+      <c r="BG22">
+        <v>13043068</v>
+      </c>
+      <c r="BH22">
+        <v>382608</v>
+      </c>
+      <c r="BI22">
+        <v>238203</v>
+      </c>
+      <c r="BJ22" s="6">
+        <f>BG22/BH22</f>
+        <v>34.089898799815998</v>
+      </c>
+      <c r="BK22" s="6">
+        <f>BG22/BI22</f>
+        <v>54.756102987787727</v>
+      </c>
     </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -3146,8 +4308,58 @@
       <c r="AL23" s="2">
         <v>1</v>
       </c>
+      <c r="AS23" t="s">
+        <v>52</v>
+      </c>
+      <c r="AT23" s="4">
+        <f t="shared" si="15"/>
+        <v>30300136</v>
+      </c>
+      <c r="AU23" s="4">
+        <f t="shared" si="16"/>
+        <v>68129027</v>
+      </c>
+      <c r="AV23" s="5">
+        <f t="shared" si="17"/>
+        <v>0.55525365128141346</v>
+      </c>
+      <c r="BA23" t="s">
+        <v>51</v>
+      </c>
+      <c r="BB23">
+        <v>13124199</v>
+      </c>
+      <c r="BC23">
+        <v>237135</v>
+      </c>
+      <c r="BD23">
+        <v>138534</v>
+      </c>
+      <c r="BE23" s="6">
+        <v>55.344841545954836</v>
+      </c>
+      <c r="BF23" s="6">
+        <v>94.736303001429249</v>
+      </c>
+      <c r="BG23">
+        <v>13515891</v>
+      </c>
+      <c r="BH23">
+        <v>542733</v>
+      </c>
+      <c r="BI23">
+        <v>319460</v>
+      </c>
+      <c r="BJ23" s="6">
+        <f t="shared" ref="BJ23:BJ24" si="18">BG23/BH23</f>
+        <v>24.903388959211988</v>
+      </c>
+      <c r="BK23" s="6">
+        <f t="shared" ref="BK23:BK24" si="19">BG23/BI23</f>
+        <v>42.30855506166656</v>
+      </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -3262,8 +4474,52 @@
       <c r="AL24" s="2">
         <v>1</v>
       </c>
+      <c r="AT24" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AV24" t="s">
+        <v>5</v>
+      </c>
+      <c r="BA24" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB24">
+        <v>10812056</v>
+      </c>
+      <c r="BC24">
+        <v>197023</v>
+      </c>
+      <c r="BD24">
+        <v>122727</v>
+      </c>
+      <c r="BE24" s="6">
+        <v>54.877126020819901</v>
+      </c>
+      <c r="BF24" s="6">
+        <v>88.098429848362628</v>
+      </c>
+      <c r="BG24">
+        <v>19488080</v>
+      </c>
+      <c r="BH24">
+        <v>533736</v>
+      </c>
+      <c r="BI24">
+        <v>396201</v>
+      </c>
+      <c r="BJ24" s="6">
+        <f t="shared" si="18"/>
+        <v>36.512582999835125</v>
+      </c>
+      <c r="BK24" s="6">
+        <f t="shared" si="19"/>
+        <v>49.187356922370213</v>
+      </c>
     </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -3378,8 +4634,37 @@
       <c r="AL25" s="2">
         <v>1</v>
       </c>
+      <c r="AS25" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT25" s="4">
+        <f>AVERAGE(AT21:AT23)</f>
+        <v>26660169.666666668</v>
+      </c>
+      <c r="AU25" s="4">
+        <f>AVERAGE(AU21:AU23)</f>
+        <v>72559401</v>
+      </c>
+      <c r="AV25" s="5">
+        <f t="shared" si="17"/>
+        <v>0.63257456236902132</v>
+      </c>
+      <c r="BB25" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="BC25" s="3"/>
+      <c r="BD25" s="3"/>
+      <c r="BE25" s="3"/>
+      <c r="BF25" s="3"/>
+      <c r="BG25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="BH25" s="3"/>
+      <c r="BI25" s="3"/>
+      <c r="BJ25" s="3"/>
+      <c r="BK25" s="3"/>
     </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -3494,8 +4779,51 @@
       <c r="AL26" s="2">
         <v>0.25</v>
       </c>
+      <c r="BA26" t="s">
+        <v>56</v>
+      </c>
+      <c r="BB26" s="6">
+        <f>AVERAGE(BB22:BB24)</f>
+        <v>11311156.666666666</v>
+      </c>
+      <c r="BC26" s="6">
+        <f>AVERAGE(BC22:BC24)</f>
+        <v>219559.66666666666</v>
+      </c>
+      <c r="BD26" s="6">
+        <f>AVERAGE(BD22:BD24)</f>
+        <v>128249.33333333333</v>
+      </c>
+      <c r="BE26" s="6">
+        <f>BB26/BC26</f>
+        <v>51.517461464537355</v>
+      </c>
+      <c r="BF26" s="6">
+        <f>BB26/BD26</f>
+        <v>88.19661180824852</v>
+      </c>
+      <c r="BG26" s="6">
+        <f>AVERAGE(BG22:BG24)</f>
+        <v>15349013</v>
+      </c>
+      <c r="BH26" s="6">
+        <f>AVERAGE(BH22:BH24)</f>
+        <v>486359</v>
+      </c>
+      <c r="BI26" s="6">
+        <f>AVERAGE(BI22:BI24)</f>
+        <v>317954.66666666669</v>
+      </c>
+      <c r="BJ26" s="6">
+        <f>BG26/BH26</f>
+        <v>31.5590191607434</v>
+      </c>
+      <c r="BK26" s="6">
+        <f>BG26/BI26</f>
+        <v>48.274218337205298</v>
+      </c>
     </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -3611,7 +4939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -3726,8 +5054,26 @@
       <c r="AL28" s="2">
         <v>1</v>
       </c>
+      <c r="BB28" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC28" t="s">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="s">
+        <v>47</v>
+      </c>
+      <c r="BE28" t="s">
+        <v>5</v>
+      </c>
+      <c r="BF28" t="s">
+        <v>60</v>
+      </c>
+      <c r="BG28" t="s">
+        <v>62</v>
+      </c>
     </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -3842,8 +5188,35 @@
       <c r="AL29" s="2">
         <v>0</v>
       </c>
+      <c r="BB29" t="s">
+        <v>42</v>
+      </c>
+      <c r="BC29">
+        <v>9549022</v>
+      </c>
+      <c r="BD29">
+        <v>22087724</v>
+      </c>
+      <c r="BE29" s="5">
+        <f>1-BC29/BD29</f>
+        <v>0.56767741212267953</v>
+      </c>
+      <c r="BF29">
+        <v>221415</v>
+      </c>
+      <c r="BG29">
+        <v>131684</v>
+      </c>
+      <c r="BH29">
+        <f>BC29/BF29</f>
+        <v>43.127258767472846</v>
+      </c>
+      <c r="BI29">
+        <f>BC29/BG29</f>
+        <v>72.514671486285351</v>
+      </c>
     </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:66" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -3958,9 +5331,48 @@
       <c r="AL30" s="2">
         <v>1</v>
       </c>
+      <c r="BB30" t="s">
+        <v>43</v>
+      </c>
+      <c r="BC30">
+        <v>13278260</v>
+      </c>
+      <c r="BD30">
+        <v>39806942</v>
+      </c>
+      <c r="BE30" s="5">
+        <f t="shared" ref="BE30:BE31" si="20">1-BC30/BD30</f>
+        <v>0.66643355824720218</v>
+      </c>
+    </row>
+    <row r="31" spans="1:66" x14ac:dyDescent="0.35">
+      <c r="BB31" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC31">
+        <v>3832888</v>
+      </c>
+      <c r="BD31">
+        <v>10664735</v>
+      </c>
+      <c r="BE31" s="5">
+        <f t="shared" si="20"/>
+        <v>0.6406016652078087</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="18">
+    <mergeCell ref="AS15:AY15"/>
+    <mergeCell ref="AZ15:BF15"/>
+    <mergeCell ref="BB20:BF20"/>
+    <mergeCell ref="BG20:BK20"/>
+    <mergeCell ref="BB25:BF25"/>
+    <mergeCell ref="BG25:BK25"/>
+    <mergeCell ref="AS3:AY3"/>
+    <mergeCell ref="AZ3:BF3"/>
+    <mergeCell ref="AQ5:AQ7"/>
+    <mergeCell ref="AQ8:AQ10"/>
+    <mergeCell ref="AQ11:AQ13"/>
     <mergeCell ref="AH1:AL1"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="I1:M1"/>

</xml_diff>